<commit_message>
some manual test cases
</commit_message>
<xml_diff>
--- a/docs/HotelTestCases.xlsx
+++ b/docs/HotelTestCases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\hotel-recommendation\hotel-recommendation\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39565FC0-1A65-4742-9CBE-CEB8AA475287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37E595C-15A3-43A6-95BF-41CA0E721F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{EEC86342-3E0E-43FC-97B5-2F7722E10954}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="60">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Expected Results</t>
   </si>
   <si>
-    <t>Actual Test</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
     <t>Atleast 1 hotel exists</t>
   </si>
   <si>
-    <t>Area: Dwarka, New Delhi</t>
-  </si>
-  <si>
     <t>Only hotels in Dwarka displayed</t>
   </si>
   <si>
@@ -90,15 +84,6 @@
     <t>TC_HOTEL_2</t>
   </si>
   <si>
-    <t>Filter by ratings</t>
-  </si>
-  <si>
-    <t>Hotel exist with ratings</t>
-  </si>
-  <si>
-    <t>Rating: ≥4</t>
-  </si>
-  <si>
     <t>Only hotels with rating ≥4 displayed</t>
   </si>
   <si>
@@ -117,73 +102,132 @@
     <t>Hotels satisfy both filters</t>
   </si>
   <si>
+    <t>TC_REV_1</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>Verify sentiment of positive review</t>
+  </si>
+  <si>
+    <t>Hotel exists with preloaded reviews</t>
+  </si>
+  <si>
+    <t>1. Select area and minimum rating            2. Click Get Recommendation</t>
+  </si>
+  <si>
+    <t>"excellent attention friendly staff very good services in general excellent wi fi and great breakfast" - from dataset</t>
+  </si>
+  <si>
+    <t>Review is labelled as positive</t>
+  </si>
+  <si>
+    <t>Sentiment shown as positive</t>
+  </si>
+  <si>
+    <t>TC_REV_2</t>
+  </si>
+  <si>
+    <t>Verify sentiment of negative review</t>
+  </si>
+  <si>
+    <t>"there are so many mosquitoes in the room" - from dataset</t>
+  </si>
+  <si>
+    <t>Review is labelled as negative</t>
+  </si>
+  <si>
+    <t>Sentiment shown as negative</t>
+  </si>
+  <si>
+    <t>TC_REV_3</t>
+  </si>
+  <si>
+    <t>Verify sentiment of neutral review</t>
+  </si>
+  <si>
+    <t>"brkfast was decent view was okayish" - from dataset</t>
+  </si>
+  <si>
+    <t>Review is labelled as neutral</t>
+  </si>
+  <si>
+    <t>Sentiment shown as neutral</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area: Dwarka, New Delhi    Rating: 7  </t>
+  </si>
+  <si>
+    <t>Filter by minimum rating</t>
+  </si>
+  <si>
+    <t>Hotel exist with rating meeting the minimim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area: Dwarka, New Delhi    Rating: 8 </t>
+  </si>
+  <si>
+    <t>Only hotels with rating ≥8 (out of 10) displayed</t>
+  </si>
+  <si>
+    <t>TC_HOTEL_4</t>
+  </si>
+  <si>
+    <t>Rating above max (&gt;10)</t>
+  </si>
+  <si>
+    <t>App is loaded on recommendation page</t>
+  </si>
+  <si>
     <t>1. Go to recommendation page
-2. Insert Minimum Rating 
-3. Click Get Recommendation</t>
-  </si>
-  <si>
-    <t>1. Select area
-2. Select rating
-3. Click Get Recommendation</t>
+2. Select area                  3. Insert Rating
+4. Click Get Recommendation</t>
   </si>
   <si>
     <t>1. Go to recommendation page
-2. Select area filter
-3. Click Get Recommendation</t>
-  </si>
-  <si>
-    <t>TC_REV_1</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>Verify sentiment of positive review</t>
-  </si>
-  <si>
-    <t>Hotel exists with preloaded reviews</t>
-  </si>
-  <si>
-    <t>1. Select area and minimum rating            2. Click Get Recommendation</t>
-  </si>
-  <si>
-    <t>"excellent attention friendly staff very good services in general excellent wi fi and great breakfast" - from dataset</t>
-  </si>
-  <si>
-    <t>Review is labelled as positive</t>
-  </si>
-  <si>
-    <t>Sentiment shown as positive</t>
-  </si>
-  <si>
-    <t>TC_REV_2</t>
-  </si>
-  <si>
-    <t>Verify sentiment of negative review</t>
-  </si>
-  <si>
-    <t>"there are so many mosquitoes in the room" - from dataset</t>
-  </si>
-  <si>
-    <t>Review is labelled as negative</t>
-  </si>
-  <si>
-    <t>Sentiment shown as negative</t>
-  </si>
-  <si>
-    <t>TC_REV_3</t>
-  </si>
-  <si>
-    <t>Verify sentiment of neutral review</t>
-  </si>
-  <si>
-    <t>"brkfast was decent view was okayish" - from dataset</t>
-  </si>
-  <si>
-    <t>Review is labelled as neutral</t>
-  </si>
-  <si>
-    <t>Sentiment shown as neutral</t>
+2. Select area                  3. Insert Rating Value above 10 (here, 111)
+4. Click Get Recommendation</t>
+  </si>
+  <si>
+    <t>Validation message shown: "Value must be less than or equal to 10"</t>
+  </si>
+  <si>
+    <t>TC_HOTEL_5</t>
+  </si>
+  <si>
+    <t>Area not selected</t>
+  </si>
+  <si>
+    <t>1. Go to recommendation page
+2. Leave area as "Choose Area"
+3. Enter a rating
+4. Click Get Recommendation</t>
+  </si>
+  <si>
+    <t>TC_HOTEL_6</t>
+  </si>
+  <si>
+    <t>Minimum rating of 0</t>
+  </si>
+  <si>
+    <t>1. Go to recommendation page
+2. Select area from dropdown
+3. Enter rating value of 0
+4. Click Get Recommendation</t>
+  </si>
+  <si>
+    <t>Area: East Delhi, New Delhi
+Rating: 0</t>
+  </si>
+  <si>
+    <t>All hotels in the selected area are displayed regardless of rating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All hotels in the selected area are displayed </t>
   </si>
 </sst>
 </file>
@@ -207,7 +251,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -217,6 +261,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -233,12 +283,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,219 +609,306 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC0FB029-86C4-44AA-BE5D-264900F6F8D4}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18.265625" customWidth="1"/>
     <col min="2" max="3" width="14.33203125" customWidth="1"/>
     <col min="4" max="4" width="12.86328125" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="9.06640625" customWidth="1"/>
+    <col min="6" max="6" width="17.06640625" customWidth="1"/>
     <col min="7" max="7" width="21.46484375" customWidth="1"/>
     <col min="8" max="8" width="12.53125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:9" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="99.75" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E4" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="114" x14ac:dyDescent="0.45">
+      <c r="A5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="114" x14ac:dyDescent="0.45">
+      <c r="A6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="A7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>14</v>
+      <c r="G8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="9" spans="1:9" ht="57" x14ac:dyDescent="0.45">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="C9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G4" t="s">
+      <c r="E9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="F9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="57" x14ac:dyDescent="0.45">
+      <c r="A10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="185.25" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" s="1" t="s">
+      <c r="F10" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="99.75" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+      <c r="G10" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="H10" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="99.75" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>14</v>
+      <c r="I10" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>